<commit_message>
v1.0.39: add XC_KEL_MISMATCH fixture + KEL logic test; 38/38 pass
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/xc_pub.xlsx
+++ b/test_data/fixtures/xc_pub.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,7 +615,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XC_FORMULA_MISMATCH</t>
+          <t>XC_KEL_MISMATCH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -667,7 +667,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>XC_VARIABLE_MISMATCH</t>
+          <t>XC_FORMULA_MISMATCH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>XC_NOT_IN_FIP</t>
+          <t>XC_VARIABLE_MISMATCH</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -771,10 +771,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XC_NOT_IN_EBX</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>XC_NOT_IN_FIP</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
@@ -819,19 +823,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XC_TOM_CORRECTION</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
+          <t>XC_NOT_IN_EBX</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>+</t>
@@ -875,7 +871,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>XC_THOUSANDS_CORR</t>
+          <t>XC_TOM_CORRECTION</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -883,7 +879,11 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>+</t>
@@ -899,7 +899,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -927,19 +927,15 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>XC_REORDER_MATCH</t>
+          <t>XC_THOUSANDS_CORR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A_ACC</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>+</t>
@@ -955,7 +951,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -988,12 +984,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B_ACC</t>
+          <t>A_ACC</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1039,11 +1035,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GB_MATCHED</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+          <t>XC_REORDER_MATCH</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B_ACC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>+</t>
@@ -1067,11 +1071,7 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>GB_GROUPING_ITEM</t>
-        </is>
-      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
@@ -1091,7 +1091,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GB_NOT_IN_FIP</t>
+          <t>GB_MATCHED</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AP_MATCH</t>
+          <t>GB_NOT_IN_FIP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1171,13 +1171,13 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>GB_GROUPING_ITEM</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
+      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AP_MISMATCH</t>
+          <t>AP_MATCH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1247,7 +1247,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>COND_MATCHED</t>
+          <t>AP_MISMATCH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1277,12 +1277,12 @@
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -1299,7 +1299,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COND_NOT_MATCHED</t>
+          <t>COND_MATCHED</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1332,7 +1332,7 @@
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
@@ -1351,7 +1351,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COND_REF_XCHECK</t>
+          <t>COND_NOT_MATCHED</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1380,15 +1380,11 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>COND_BASE</t>
-        </is>
-      </c>
+      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
@@ -1407,14 +1403,10 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XC_DIFF_IN_SCOPE</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>COND_REF_XCHECK</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
@@ -1440,9 +1432,17 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>COND_BASE</t>
+        </is>
+      </c>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -1451,11 +1451,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
+      <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
@@ -1463,7 +1459,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XC_DIFF_EXCLUDED</t>
+          <t>XC_DIFF_IN_SCOPE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1512,21 +1508,21 @@
           <t>Changed</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>COND_DIFF_YELLOW</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
+          <t>XC_DIFF_EXCLUDED</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
@@ -1554,11 +1550,7 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
-      <c r="R20" s="1" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -1567,15 +1559,23 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>COND_DIFF_GREEN</t>
+          <t>COND_DIFF_YELLOW</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1606,7 +1606,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr">
+      <c r="R21" s="1" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
@@ -1627,7 +1627,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COND_DIFF_WHITE</t>
+          <t>COND_DIFF_GREEN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1658,7 +1658,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
@@ -1676,6 +1676,58 @@
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>COND_DIFF_WHITE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.0.41: comprehensive XC fixtures (26 rows, all transform paths); KEL fingerprint no-match test; 58/58 pass
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/xc_pub.xlsx
+++ b/test_data/fixtures/xc_pub.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,7 +615,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>XC_KEL_MISMATCH</t>
+          <t>XC_ALL_MISMATCH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>XC_THOUSANDS_CORR</t>
+          <t>XC_REX_CORRECTION</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -935,7 +935,11 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>+</t>
@@ -951,7 +955,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -979,19 +983,15 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>XC_REORDER_MATCH</t>
+          <t>XC_THOUSANDS_CORR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A_ACC</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>+</t>
@@ -1007,7 +1007,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1040,12 +1040,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B_ACC</t>
+          <t>A_ACC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1091,11 +1091,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GB_MATCHED</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+          <t>XC_REORDER_MATCH</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B_ACC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>+</t>
@@ -1119,11 +1127,7 @@
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>GB_GROUPING_ITEM</t>
-        </is>
-      </c>
+      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
@@ -1143,10 +1147,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GB_NOT_IN_FIP</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>XC_ABS_FORMULA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
@@ -1160,22 +1168,26 @@
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>GB_GROUPING_ITEM</t>
-        </is>
-      </c>
+      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
@@ -1195,10 +1207,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AP_MATCH</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>XC_LC_YTD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
@@ -1206,7 +1222,11 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Shareholders' Equity</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -1225,11 +1245,7 @@
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
+      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
@@ -1247,10 +1263,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AP_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
+          <t>XC_LC_CONST</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
@@ -1258,7 +1278,11 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Shareholders' Equity</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -1267,7 +1291,7 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1277,11 +1301,7 @@
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
+      <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
@@ -1299,10 +1319,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>COND_MATCHED</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>XC_PCT_FORMAT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
@@ -1313,28 +1337,28 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>&lt;=</t>
+          <t>&lt;</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -1351,10 +1375,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>COND_NOT_MATCHED</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>XC_FF_SUFFIX</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
@@ -1382,11 +1410,7 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+      <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -1403,10 +1427,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COND_REF_XCHECK</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>XC_FF_SUFFIX</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ACC002</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
@@ -1432,17 +1460,9 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>COND_BASE</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -1459,12 +1479,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XC_DIFF_IN_SCOPE</t>
+          <t>XC_SUBTRACT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ACC001</t>
+          <t>ACC_POS</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1503,11 +1523,7 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
+      <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
@@ -1515,18 +1531,18 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>XC_DIFF_EXCLUDED</t>
+          <t>XC_SUBTRACT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACC001</t>
+          <t>ACC_NEG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1559,26 +1575,22 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>COND_DIFF_YELLOW</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>XC_NONZERO_LIMIT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
@@ -1595,7 +1607,7 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1606,11 +1618,7 @@
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
-      <c r="R21" s="1" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -1627,10 +1635,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COND_DIFF_GREEN</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>XC_GTE_OPERATOR</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
@@ -1641,7 +1653,7 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>&lt;=</t>
+          <t>&gt;=</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1658,11 +1670,7 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -1679,10 +1687,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>COND_DIFF_WHITE</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+          <t>XC_EXCL_MATCH</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
@@ -1704,17 +1716,17 @@
       </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -1728,6 +1740,922 @@
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>XC_EXCL_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>XC_KEL_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>XC_KEL_NO_MATCH</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GB_MATCHED</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>GB_GROUPING_ITEM</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GB_NOT_IN_FIP</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>GB_GROUPING_ITEM</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AP_MATCH</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AP_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>COND_MATCHED</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>COND_NOT_MATCHED</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>COND_REF_XCHECK</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>COND_BASE</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>XC_DIFF_IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>XC_DIFF_EXCLUDED</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>XC_DIFF_INACTIVE</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>XC_DIFF_YELLOW_CAT</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>Test Cat</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>COND_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" s="1" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>COND_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>COND_DIFF_WHITE</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v1.0.75: consolidated flat fixture layout; GCoA test; 149 assertions all pass
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/xc_pub.xlsx
+++ b/test_data/fixtures/xc_pub.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z44"/>
+  <dimension ref="A1:AC75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,6 +563,21 @@
       <c r="Z1" t="inlineStr">
         <is>
           <t>In Scope</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Stammhaus SLST RFD</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Stammhaus SLST SFD</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>IFRS New SFD</t>
         </is>
       </c>
     </row>
@@ -617,6 +632,9 @@
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -669,6 +687,9 @@
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -721,6 +742,9 @@
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -773,6 +797,9 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -825,6 +852,9 @@
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -873,6 +903,9 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -929,6 +962,9 @@
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -985,6 +1021,9 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1037,6 +1076,9 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1093,6 +1135,9 @@
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1149,6 +1194,9 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1209,6 +1257,9 @@
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1265,6 +1316,9 @@
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1321,6 +1375,9 @@
       <c r="X15" t="inlineStr"/>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1377,6 +1434,9 @@
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1429,6 +1489,9 @@
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1481,6 +1544,9 @@
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1533,6 +1599,9 @@
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1585,6 +1654,9 @@
       <c r="X20" t="inlineStr"/>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1637,6 +1709,9 @@
       <c r="X21" t="inlineStr"/>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1689,6 +1764,9 @@
       <c r="X22" t="inlineStr"/>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1745,6 +1823,9 @@
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1801,16 +1882,19 @@
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>XC_KEL_MISMATCH</t>
+          <t>XC_QU_YTD</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ACC001</t>
+          <t>ACC_QU</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1853,11 +1937,14 @@
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>XC_KEL_NO_MATCH</t>
+          <t>XC_KEL_MISMATCH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1905,14 +1992,21 @@
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GB_MATCHED</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>XC_KEL_NO_MATCH</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
@@ -1937,11 +2031,7 @@
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>GB_GROUPING_ITEM</t>
-        </is>
-      </c>
+      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
@@ -1957,14 +2047,21 @@
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GB_NOT_IN_FIP</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>XC_DIFF_IN_SCOPE</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
@@ -1989,11 +2086,7 @@
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>GB_GROUPING_ITEM</t>
-        </is>
-      </c>
+      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
@@ -2005,18 +2098,29 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W28" t="inlineStr"/>
+      <c r="W28" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AP_MATCH</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>XC_DIFF_EXCLUDED</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
@@ -2043,11 +2147,7 @@
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
+      <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
@@ -2057,18 +2157,33 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
+      <c r="W29" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AP_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>XC_DIFF_INACTIVE</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
@@ -2095,32 +2210,39 @@
       <c r="N30" t="inlineStr"/>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>w</t>
-        </is>
-      </c>
+      <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr"/>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="W30" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>COND_MATCHED</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>XC_DIFF_YELLOW_CAT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
@@ -2128,7 +2250,11 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" s="1" t="inlineStr">
+        <is>
+          <t>Test Cat</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -2148,11 +2274,7 @@
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
@@ -2161,18 +2283,29 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W31" t="inlineStr"/>
+      <c r="W31" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COND_NOT_MATCHED</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>XC_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
@@ -2200,11 +2333,7 @@
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
+      <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
@@ -2213,18 +2342,29 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W32" t="inlineStr"/>
+      <c r="W32" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>COND_REF_XCHECK</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t>XC_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ACC001</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
@@ -2250,17 +2390,9 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
       <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>COND_BASE</t>
-        </is>
-      </c>
+      <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
@@ -2269,15 +2401,22 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W33" t="inlineStr"/>
+      <c r="W33" s="2" t="inlineStr">
+        <is>
+          <t>New x-check or association</t>
+        </is>
+      </c>
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>XC_DIFF_IN_SCOPE</t>
+          <t>XC_DIFF_ORANGE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2321,19 +2460,22 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W34" s="1" t="inlineStr">
-        <is>
-          <t>Changed</t>
+      <c r="W34" s="3" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>XC_DIFF_EXCLUDED</t>
+          <t>XC_DIFF_NO_TOC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2377,30 +2519,21 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W35" s="1" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>XC_DIFF_INACTIVE</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_MATCHED</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
@@ -2425,7 +2558,11 @@
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
@@ -2434,29 +2571,24 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>INACTIVE</t>
-        </is>
-      </c>
-      <c r="W36" s="1" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>XC_DIFF_YELLOW_CAT</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_NOT_IN_FIP</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
@@ -2464,11 +2596,7 @@
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" s="1" t="inlineStr">
-        <is>
-          <t>Test Cat</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>&lt;=</t>
@@ -2485,7 +2613,11 @@
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
@@ -2497,26 +2629,21 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W37" s="1" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
+      <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>XC_DIFF_YELLOW</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_REF_XC_KEY</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
@@ -2541,8 +2668,16 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>REF_BASE</t>
+        </is>
+      </c>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2553,26 +2688,21 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W38" s="1" t="inlineStr">
-        <is>
-          <t>Changed</t>
-        </is>
-      </c>
+      <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>XC_DIFF_GREEN</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_MULTI</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
@@ -2597,7 +2727,11 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>ITEM_A, ITEM_B</t>
+        </is>
+      </c>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
@@ -2609,26 +2743,21 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W39" s="2" t="inlineStr">
-        <is>
-          <t>New x-check or association</t>
-        </is>
-      </c>
+      <c r="W39" t="inlineStr"/>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>XC_DIFF_ORANGE</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_DEDUP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
@@ -2653,7 +2782,11 @@
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
@@ -2665,26 +2798,21 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="W40" s="3" t="inlineStr">
-        <is>
-          <t>Removed</t>
-        </is>
-      </c>
+      <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>XC_DIFF_NO_TOC</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>ACC001</t>
-        </is>
-      </c>
+          <t>GB_DEDUP</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
@@ -2709,7 +2837,11 @@
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>ITEM_B</t>
+        </is>
+      </c>
       <c r="P41" t="inlineStr"/>
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
@@ -2725,11 +2857,14 @@
       <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>COND_DIFF_YELLOW</t>
+          <t>GB_IGNORE_FIELD</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
@@ -2757,14 +2892,14 @@
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
-      <c r="R42" s="1" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
@@ -2777,11 +2912,14 @@
       <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>COND_DIFF_GREEN</t>
+          <t>GB_UNMAPPED</t>
         </is>
       </c>
       <c r="B43" t="inlineStr"/>
@@ -2809,14 +2947,14 @@
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
-      <c r="R43" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
@@ -2829,11 +2967,14 @@
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>COND_DIFF_WHITE</t>
+          <t>GB_BLANK_VR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr"/>
@@ -2861,14 +3002,14 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr"/>
       <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr"/>
@@ -2881,6 +3022,1734 @@
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>GB_KEL_MATCH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GB_KEL_NO_MATCH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>GB_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" s="1" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GB_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W48" t="inlineStr"/>
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
+      <c r="Z48" t="inlineStr"/>
+      <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
+      <c r="AC48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>GB_DIFF_WHITE</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>ITEM_A</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
+      <c r="Z49" t="inlineStr"/>
+      <c r="AA49" t="inlineStr"/>
+      <c r="AB49" t="inlineStr"/>
+      <c r="AC49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>AP_MATCH_W</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr"/>
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
+      <c r="Z50" t="inlineStr"/>
+      <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
+      <c r="AC50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AP_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
+      <c r="Z51" t="inlineStr"/>
+      <c r="AA51" t="inlineStr"/>
+      <c r="AB51" t="inlineStr"/>
+      <c r="AC51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AP_BOTH_W</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
+      <c r="Z52" t="inlineStr"/>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr"/>
+      <c r="AC52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>AP_BOTH_E</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
+      <c r="Z53" t="inlineStr"/>
+      <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="AC53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AP_GREY_WINS</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr"/>
+      <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
+      <c r="Z54" t="inlineStr"/>
+      <c r="AA54" t="inlineStr"/>
+      <c r="AB54" t="inlineStr"/>
+      <c r="AC54" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>AP_NO_BINDING</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr"/>
+      <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
+      <c r="Z55" t="inlineStr"/>
+      <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
+      <c r="AC55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>AP_NO_ACTUAL</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr"/>
+      <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
+      <c r="Z56" t="inlineStr"/>
+      <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
+      <c r="AC56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AP_NOT_SCOPE_TOC</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr"/>
+      <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
+      <c r="Z57" t="inlineStr"/>
+      <c r="AA57" t="inlineStr"/>
+      <c r="AB57" t="inlineStr"/>
+      <c r="AC57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>AP_NOT_SCOPE_INA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr"/>
+      <c r="X58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr"/>
+      <c r="Z58" t="inlineStr"/>
+      <c r="AA58" t="inlineStr"/>
+      <c r="AB58" t="inlineStr"/>
+      <c r="AC58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>AP_EXCL_ZCORE</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr"/>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr"/>
+      <c r="Z59" t="inlineStr"/>
+      <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
+      <c r="AC59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>AP_YELLOW_CAT</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" s="1" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr"/>
+      <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
+      <c r="Z60" t="inlineStr"/>
+      <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
+      <c r="AC60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>AP_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" s="1" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W61" s="1" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
+      <c r="Z61" t="inlineStr"/>
+      <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
+      <c r="AC61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>AP_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr"/>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W62" s="2" t="inlineStr">
+        <is>
+          <t>New x-check or association</t>
+        </is>
+      </c>
+      <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
+      <c r="Z62" t="inlineStr"/>
+      <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
+      <c r="AC62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>AP_DIFF_WHITE</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr"/>
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr"/>
+      <c r="Z63" t="inlineStr"/>
+      <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
+      <c r="AC63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>COND_APPL_QTRS</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr"/>
+      <c r="Z64" t="inlineStr"/>
+      <c r="AA64" t="inlineStr"/>
+      <c r="AB64" t="inlineStr"/>
+      <c r="AC64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>COND_INCL_RUS</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>RU_NORTH</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr"/>
+      <c r="U65" t="inlineStr"/>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr"/>
+      <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr"/>
+      <c r="Z65" t="inlineStr"/>
+      <c r="AA65" t="inlineStr"/>
+      <c r="AB65" t="inlineStr"/>
+      <c r="AC65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>COND_EXCL_RUS</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>RU_SOUTH</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr"/>
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
+      <c r="Z66" t="inlineStr"/>
+      <c r="AA66" t="inlineStr"/>
+      <c r="AB66" t="inlineStr"/>
+      <c r="AC66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>COND_LIMIT_PCT</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>10.5</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr"/>
+      <c r="X67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr"/>
+      <c r="Z67" t="inlineStr"/>
+      <c r="AA67" t="inlineStr"/>
+      <c r="AB67" t="inlineStr"/>
+      <c r="AC67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>COND_NOT_MATCHED</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr"/>
+      <c r="X68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr"/>
+      <c r="Z68" t="inlineStr"/>
+      <c r="AA68" t="inlineStr"/>
+      <c r="AB68" t="inlineStr"/>
+      <c r="AC68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>COND_MULTI_COL</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>RU_IN</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>RU_OUT</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr"/>
+      <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr"/>
+      <c r="Z69" t="inlineStr"/>
+      <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
+      <c r="AC69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>COND_KEL_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr"/>
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
+      <c r="Z70" t="inlineStr"/>
+      <c r="AA70" t="inlineStr"/>
+      <c r="AB70" t="inlineStr"/>
+      <c r="AC70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>COND_KEL_NO_MATCH</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr"/>
+      <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr"/>
+      <c r="Z71" t="inlineStr"/>
+      <c r="AA71" t="inlineStr"/>
+      <c r="AB71" t="inlineStr"/>
+      <c r="AC71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>COND_REF_XC</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>COND_REF_XC</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr"/>
+      <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr"/>
+      <c r="Z72" t="inlineStr"/>
+      <c r="AA72" t="inlineStr"/>
+      <c r="AB72" t="inlineStr"/>
+      <c r="AC72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>COND_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" s="1" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr"/>
+      <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
+      <c r="Z73" t="inlineStr"/>
+      <c r="AA73" t="inlineStr"/>
+      <c r="AB73" t="inlineStr"/>
+      <c r="AC73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>COND_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" s="2" t="inlineStr">
+        <is>
+          <t>RU_NORTH</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr"/>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr"/>
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
+      <c r="Z74" t="inlineStr"/>
+      <c r="AA74" t="inlineStr"/>
+      <c r="AB74" t="inlineStr"/>
+      <c r="AC74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>COND_DIFF_WHITE</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>&lt;=</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr"/>
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr"/>
+      <c r="Z75" t="inlineStr"/>
+      <c r="AA75" t="inlineStr"/>
+      <c r="AB75" t="inlineStr"/>
+      <c r="AC75" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>